<commit_message>
Remove hardcoded agenda data and enforce MongoDB as single source of truth
</commit_message>
<xml_diff>
--- a/IEEE Deeptech.ai Agenda.xlsx
+++ b/IEEE Deeptech.ai Agenda.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
   <si>
     <t>Time</t>
   </si>
@@ -22,13 +22,25 @@
     <t>Sub-Topic / Focus Area / Panel Details</t>
   </si>
   <si>
-    <t>8.30 - 10am</t>
-  </si>
-  <si>
-    <t>Opening Keynote: The Dawn of Physical AI</t>
+    <t>8.30 - 9.30am</t>
+  </si>
+  <si>
+    <t>Networking</t>
   </si>
   <si>
     <t>Bridging Foundation Models, World Models, and Spatial Computing</t>
+  </si>
+  <si>
+    <t>9.30 - 9.45 am</t>
+  </si>
+  <si>
+    <t>Opening/Inaugral</t>
+  </si>
+  <si>
+    <t>9.45 - 10am</t>
+  </si>
+  <si>
+    <t>Keynote GE Site Head</t>
   </si>
   <si>
     <t>10:00 - 10:30</t>
@@ -64,9 +76,6 @@
   </si>
   <si>
     <t>12:15 - 12:30</t>
-  </si>
-  <si>
-    <t>Networking</t>
   </si>
   <si>
     <t xml:space="preserve"> Lounge, Photo Booth</t>
@@ -117,22 +126,7 @@
 • Research vs. Industry roles, higher studies, and startup founding</t>
   </si>
   <si>
-    <t>16:00 - 16:30</t>
-  </si>
-  <si>
-    <t>Agentic Control in Embedded Systems OR Combining LLM Reasoners with Low-Latency Motion Planning</t>
-  </si>
-  <si>
-    <t>16:30 - 17:00</t>
-  </si>
-  <si>
-    <t>Founders &amp; Researchers Spotlight: Frontier Innovations</t>
-  </si>
-  <si>
-    <t>Highlighting Breakthrough Startups in Embodied &amp; Physical AI</t>
-  </si>
-  <si>
-    <t>17:00 - 17:15</t>
+    <t>16:00 - 16.15</t>
   </si>
   <si>
     <t>Closing Remarks &amp; Future Outlook</t>
@@ -204,7 +198,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -218,6 +212,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -435,7 +432,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="10.88"/>
+    <col customWidth="1" min="1" max="1" width="18.13"/>
     <col customWidth="1" min="2" max="2" width="78.88"/>
     <col customWidth="1" min="3" max="3" width="54.38"/>
   </cols>
@@ -469,27 +466,27 @@
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>8</v>
-      </c>
+      <c r="C4" s="3"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="4"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="4"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
@@ -498,113 +495,126 @@
       <c r="B7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="C7" s="4"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>18</v>
-      </c>
+      <c r="C8" s="4"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" s="4"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="4"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>25</v>
-      </c>
+      <c r="C11" s="4"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>27</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="C12" s="4"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>32</v>
+      <c r="C14" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15" s="4"/>
+        <v>31</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="3" t="s">
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="B17" s="3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="s">
+      <c r="C17" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>40</v>
-      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="4"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>